<commit_message>
fixes to align new real test
</commit_message>
<xml_diff>
--- a/tests/real2/planner.xlsx
+++ b/tests/real2/planner.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dev/Desktop/busplan/tests/real2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBF3171-EBA1-204D-B015-D0435731CCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF679DA-9D5F-954C-89B4-00B4EC3B236D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="860" yWindow="500" windowWidth="27240" windowHeight="14980" xr2:uid="{C9FFF9DD-589D-764B-815C-08A9278F4BF4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="78">
   <si>
     <t>Bus</t>
   </si>
@@ -77,9 +77,6 @@
     <t>IC Cembra</t>
   </si>
   <si>
-    <t>IC Civezzano</t>
-  </si>
-  <si>
     <t>Bus 5</t>
   </si>
   <si>
@@ -189,9 +186,6 @@
   </si>
   <si>
     <t xml:space="preserve">Via Negritelle, 1, Cembra (TN) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Via Murialdo, 27, Civezzano (TN) </t>
   </si>
   <si>
     <t xml:space="preserve">Piazza Brenta Alta, Madonna di Campiglio (TN) </t>
@@ -663,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA9D099C-0CAE-254A-9309-2CE31771A950}">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
@@ -678,13 +672,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -699,7 +693,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D2" s="2">
         <v>18</v>
@@ -715,7 +709,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D3" s="2">
         <v>30</v>
@@ -731,7 +725,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="2">
         <v>22</v>
@@ -747,7 +741,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D5" s="2">
         <v>31</v>
@@ -763,7 +757,7 @@
         <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" s="2">
         <v>26</v>
@@ -779,7 +773,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7" s="2">
         <v>18</v>
@@ -795,7 +789,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D8" s="2">
         <v>23</v>
@@ -805,48 +799,48 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D9" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="3"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D10" s="2">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="3"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="2">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="3"/>
@@ -856,336 +850,320 @@
         <v>18</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="D12" s="2">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>56</v>
       </c>
       <c r="D13" s="2">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="D14" s="2">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D15" s="2">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="D16" s="2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D17" s="2">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D18" s="2">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="D19" s="2">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D20" s="2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="D21" s="2">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D22" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="3"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>68</v>
       </c>
       <c r="D23" s="2">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="3"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="D24" s="2">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="3"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D25" s="2">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="3"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D26" s="2">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" s="3"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D27" s="2">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="3"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D28" s="2">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="3"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>37</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D29" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" s="3"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D30" s="2">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" s="3"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D31" s="2">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" s="3"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D32" s="2">
-        <v>32</v>
-      </c>
-      <c r="E32" s="2"/>
-      <c r="F32" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>